<commit_message>
Barre de recherche Et documentation
</commit_message>
<xml_diff>
--- a/doc/Planification.xlsx
+++ b/doc/Planification.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ilan.mlq\Documents\Ecole\Wiki-Cars\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEA0DE7B-19D6-487F-A94D-92824B0A9583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{129FEB3E-25E6-46AB-8049-70626377764E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planning prévisionnel" sheetId="1" r:id="rId1"/>
     <sheet name="Planning effectif" sheetId="2" r:id="rId2"/>
-    <sheet name="Exemple" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="53">
   <si>
     <t>Tâches à réaliser</t>
   </si>
@@ -88,55 +87,7 @@
     <t>Page de deconnexion</t>
   </si>
   <si>
-    <t>Page des annonces personnelles</t>
-  </si>
-  <si>
     <t>Page d'administration</t>
-  </si>
-  <si>
-    <t>Page des articles</t>
-  </si>
-  <si>
-    <t>Page des catégories</t>
-  </si>
-  <si>
-    <t>Page d'ajout d'article</t>
-  </si>
-  <si>
-    <t>Page de modification d'article</t>
-  </si>
-  <si>
-    <t>Afficher Annonces + commentaires</t>
-  </si>
-  <si>
-    <t>Afficher catégories</t>
-  </si>
-  <si>
-    <t>Rechercher annonces</t>
-  </si>
-  <si>
-    <t>Ajouter Annonce</t>
-  </si>
-  <si>
-    <t>Ajouter Commentaire</t>
-  </si>
-  <si>
-    <t>Connexion</t>
-  </si>
-  <si>
-    <t>deconnexion</t>
-  </si>
-  <si>
-    <t>Modification Annonces</t>
-  </si>
-  <si>
-    <t>suppression Annonces</t>
-  </si>
-  <si>
-    <t>Ajoute/enleve des catégories</t>
-  </si>
-  <si>
-    <t>Relancer une annonce</t>
   </si>
   <si>
     <t>Documentation</t>
@@ -161,9 +112,6 @@
   </si>
   <si>
     <t>GENERAL</t>
-  </si>
-  <si>
-    <t>Test et débogage</t>
   </si>
   <si>
     <t>MCD</t>
@@ -239,6 +187,15 @@
   </si>
   <si>
     <t>Test</t>
+  </si>
+  <si>
+    <t>Type de transmission</t>
+  </si>
+  <si>
+    <t>Type de boite de vitesse</t>
+  </si>
+  <si>
+    <t>Barre de recherche</t>
   </si>
 </sst>
 </file>
@@ -520,24 +477,36 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="74">
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
+  <dxfs count="73">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
         </patternFill>
       </fill>
     </dxf>
@@ -570,6 +539,17 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="none"/>
       </fill>
@@ -584,6 +564,46 @@
     </dxf>
     <dxf>
       <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6D9F0"/>
           <bgColor rgb="FFC6D9F0"/>
@@ -591,6 +611,40 @@
       </fill>
     </dxf>
     <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFB8CCE4"/>
+          <bgColor rgb="FFB8CCE4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <font>
         <color rgb="FF9C0006"/>
       </font>
@@ -609,8 +663,16 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -623,6 +685,110 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFC6D9F0"/>
+          <bgColor rgb="FFC6D9F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFB8CCE4"/>
@@ -631,10 +797,12 @@
       </fill>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -669,234 +837,7 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFB8CCE4"/>
-          <bgColor rgb="FFB8CCE4"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFC6D9F0"/>
-          <bgColor rgb="FFC6D9F0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="none"/>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
       </fill>
     </dxf>
     <dxf>
@@ -1521,7 +1462,7 @@
     </row>
     <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="36" t="s">
-        <v>35</v>
+        <v>19</v>
       </c>
       <c r="B2" s="6">
         <v>4.1666666666666664E-2</v>
@@ -1546,7 +1487,7 @@
     </row>
     <row r="3" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="37" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="B3" s="29">
         <v>8.3333333333333329E-2</v>
@@ -1571,7 +1512,7 @@
     </row>
     <row r="4" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="37" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B4" s="29">
         <v>4.1666666666666664E-2</v>
@@ -1596,7 +1537,7 @@
     </row>
     <row r="5" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="23" t="s">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="B5" s="24"/>
       <c r="C5" s="25"/>
@@ -1613,8 +1554,8 @@
       <c r="N5" s="10"/>
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="39" t="s">
-        <v>36</v>
+      <c r="A6" s="38" t="s">
+        <v>20</v>
       </c>
       <c r="B6" s="29">
         <v>8.3333333333333329E-2</v>
@@ -1690,7 +1631,7 @@
     </row>
     <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="B9" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1714,7 +1655,7 @@
     </row>
     <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B10" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1739,7 +1680,7 @@
     </row>
     <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="B11" s="11">
         <v>8.3333333333333329E-2</v>
@@ -1766,7 +1707,7 @@
     </row>
     <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
-        <v>64</v>
+        <v>47</v>
       </c>
       <c r="B12" s="11">
         <v>8.3333333333333329E-2</v>
@@ -1791,7 +1732,7 @@
     </row>
     <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="23" t="s">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="B13" s="24"/>
       <c r="C13" s="28"/>
@@ -1809,7 +1750,7 @@
     </row>
     <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="37" t="s">
-        <v>43</v>
+        <v>26</v>
       </c>
       <c r="B14" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1834,7 +1775,7 @@
     </row>
     <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
-        <v>44</v>
+        <v>27</v>
       </c>
       <c r="B15" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1861,7 +1802,7 @@
     </row>
     <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
-        <v>45</v>
+        <v>28</v>
       </c>
       <c r="B16" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1886,7 +1827,7 @@
     </row>
     <row r="17" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="B17" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1911,7 +1852,7 @@
     </row>
     <row r="18" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="37" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B18" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1935,7 +1876,7 @@
     </row>
     <row r="19" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="37" t="s">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="B19" s="11">
         <v>4.1666666666666664E-2</v>
@@ -1959,7 +1900,7 @@
     </row>
     <row r="20" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="37" t="s">
-        <v>49</v>
+        <v>32</v>
       </c>
       <c r="B20" s="11">
         <v>8.3333333333333329E-2</v>
@@ -1983,7 +1924,7 @@
     </row>
     <row r="21" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
-        <v>50</v>
+        <v>33</v>
       </c>
       <c r="B21" s="29">
         <v>0.125</v>
@@ -2009,7 +1950,7 @@
     </row>
     <row r="22" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="37" t="s">
-        <v>52</v>
+        <v>35</v>
       </c>
       <c r="B22" s="29">
         <v>6.25E-2</v>
@@ -2033,7 +1974,7 @@
     </row>
     <row r="23" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="37" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
       <c r="B23" s="29">
         <v>8.3333333333333329E-2</v>
@@ -2057,7 +1998,7 @@
     </row>
     <row r="24" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="37" t="s">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="B24" s="29">
         <v>8.3333333333333329E-2</v>
@@ -2084,7 +2025,7 @@
     </row>
     <row r="25" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="37" t="s">
-        <v>53</v>
+        <v>36</v>
       </c>
       <c r="B25" s="29">
         <v>6.25E-2</v>
@@ -2109,7 +2050,7 @@
     </row>
     <row r="26" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="37" t="s">
-        <v>55</v>
+        <v>38</v>
       </c>
       <c r="B26" s="29">
         <v>8.3333333333333329E-2</v>
@@ -2135,7 +2076,7 @@
     </row>
     <row r="27" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="37" t="s">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="B27" s="29">
         <v>8.3333333333333329E-2</v>
@@ -2158,7 +2099,7 @@
     </row>
     <row r="28" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="37" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="B28" s="11">
         <v>8.3333333333333329E-2</v>
@@ -2182,7 +2123,7 @@
     </row>
     <row r="29" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="37" t="s">
-        <v>58</v>
+        <v>41</v>
       </c>
       <c r="B29" s="11">
         <v>8.3333333333333329E-2</v>
@@ -2205,7 +2146,7 @@
     </row>
     <row r="30" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="37" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="B30" s="29">
         <v>8.3333333333333329E-2</v>
@@ -2230,7 +2171,7 @@
     </row>
     <row r="31" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="37" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="B31" s="29">
         <v>8.3333333333333329E-2</v>
@@ -2257,7 +2198,7 @@
     </row>
     <row r="32" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="37" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="B32" s="29">
         <v>8.3333333333333329E-2</v>
@@ -2280,7 +2221,7 @@
     </row>
     <row r="33" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="23" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="B33" s="24"/>
       <c r="C33" s="28"/>
@@ -2298,7 +2239,7 @@
     </row>
     <row r="34" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="37" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="B34" s="11">
         <v>0.41666666666666669</v>
@@ -2341,7 +2282,7 @@
     </row>
     <row r="35" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="37" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="B35" s="11">
         <v>0.22916666666666666</v>
@@ -2386,7 +2327,7 @@
     </row>
     <row r="36" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="37" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="B36" s="11">
         <v>1</v>
@@ -2430,8 +2371,8 @@
       </c>
     </row>
     <row r="37" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="40" t="s">
-        <v>34</v>
+      <c r="A37" s="39" t="s">
+        <v>18</v>
       </c>
       <c r="B37" s="17">
         <v>0.10416666666666667</v>
@@ -3487,158 +3428,170 @@
     <row r="1010" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1011" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color theme="4" tint="0.59999389629810485"/>
+        <color theme="8" tint="0.39997558519241921"/>
+        <color theme="8" tint="-0.249977111117893"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="C5:C7 D8:D9 F18:F21 E22:E37 G24:H24 G25 H26 J27:J28 G27:G37 K29 I30:I33 K31">
-    <cfRule type="cellIs" dxfId="73" priority="5" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="72" priority="6" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C7 D8 D9:J9 F18:J20 F21 C22:E23 C24:J25 C26:F26 H26:J26 C27:G27 J27:J28 C28:H29 K29 C30:J31 K31 C32:I32 C33:K33 K5:M12 C14:J17 L14:M33 C18:D21 G21:J23">
-    <cfRule type="cellIs" dxfId="72" priority="24" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="71" priority="25" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C36:D36">
-    <cfRule type="cellIs" dxfId="71" priority="11" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="70" priority="12" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="69" priority="13" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="68" priority="14" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C5:J6 D7:J8">
-    <cfRule type="cellIs" dxfId="68" priority="36" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="67" priority="37" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="66" priority="38" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10:J12">
-    <cfRule type="cellIs" dxfId="66" priority="6" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="65" priority="7" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="64" priority="8" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="63" priority="9" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34:J35 L34:M37 E36:J36 K14:K31 L31:L32 C37:J37">
-    <cfRule type="cellIs" dxfId="63" priority="68" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="62" priority="69" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34:J35 L34:M37 E36:J36">
-    <cfRule type="cellIs" dxfId="62" priority="67" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="61" priority="68" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C34:K34 C35:J35 E36:J36 C37:J37 K35:K37 K14:K31 L31:L32">
-    <cfRule type="cellIs" dxfId="61" priority="62" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="60" priority="63" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:M4 K33:K37">
-    <cfRule type="cellIs" dxfId="60" priority="60" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="59" priority="61" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:M4">
-    <cfRule type="cellIs" dxfId="59" priority="53" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="58" priority="54" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="54" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="57" priority="55" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C13:M13">
-    <cfRule type="cellIs" dxfId="57" priority="2" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="56" priority="3" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
     <cfRule type="cellIs" dxfId="55" priority="4" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="54" priority="5" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C38:M38">
-    <cfRule type="cellIs" dxfId="54" priority="47" operator="equal">
+    <cfRule type="cellIs" dxfId="53" priority="48" operator="equal">
       <formula>0.333333333333333</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D34:D35 J34:J36 F36 H36 M36">
-    <cfRule type="cellIs" dxfId="53" priority="65" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="52" priority="66" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D36">
-    <cfRule type="cellIs" dxfId="52" priority="9" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="51" priority="10" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="51" priority="10" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="50" priority="11" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D7:J8 C5:J6">
-    <cfRule type="cellIs" dxfId="50" priority="35" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="49" priority="36" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:E17 G5:G23 I5:I26 L5:L37 C10:C37">
-    <cfRule type="cellIs" dxfId="49" priority="1" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="48" priority="2" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F34:F35 H34:I35 I36:I37">
-    <cfRule type="cellIs" dxfId="48" priority="61" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="47" priority="62" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G34:G35">
-    <cfRule type="cellIs" dxfId="47" priority="66" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="46" priority="67" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K14:K31 L31:L32 C34:J35 L34:M37 E36:J36 C37:J37">
-    <cfRule type="cellIs" dxfId="46" priority="69" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="45" priority="70" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K33:K37 C2:M4">
-    <cfRule type="cellIs" dxfId="45" priority="59" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="44" priority="60" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K34:K36">
-    <cfRule type="cellIs" dxfId="44" priority="56" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="43" priority="57" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5:M12 C7 D8 D9:J9 C14:J17 L14:M33 F18:J20 C18:D21 F21 G21:J23 C22:E23 C24:J25 C26:F26 H26:J26 C27:G27 J27:J28 C28:H29 K29 C30:J31 K31 C32:I32 C33:J33">
-    <cfRule type="cellIs" dxfId="43" priority="26" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="42" priority="26" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="25" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="41" priority="27" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K34:M37">
-    <cfRule type="cellIs" dxfId="41" priority="58" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="40" priority="59" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N2:N4 N6:N12 N14:N32">
-    <cfRule type="cellIs" dxfId="40" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="39" priority="52" operator="equal">
       <formula>$B2</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N34:N37">
-    <cfRule type="cellIs" dxfId="39" priority="49" operator="equal">
+    <cfRule type="cellIs" dxfId="38" priority="50" operator="equal">
       <formula>$B34</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3649,7 +3602,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:AA1002"/>
+  <dimension ref="A1:AA1003"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42.625" customWidth="1"/>
@@ -3657,7 +3610,7 @@
     <col min="3" max="27" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3700,7 +3653,6 @@
       <c r="N1" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="5"/>
       <c r="P1" s="5"/>
       <c r="Q1" s="5"/>
       <c r="R1" s="5"/>
@@ -3715,9 +3667,15 @@
       <c r="AA1" s="5"/>
     </row>
     <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="36"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="7"/>
+      <c r="A2" s="36" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="6">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="C2" s="7">
+        <v>4.1666666666666664E-2</v>
+      </c>
       <c r="D2" s="8"/>
       <c r="E2" s="7"/>
       <c r="F2" s="8"/>
@@ -3730,13 +3688,19 @@
       <c r="M2" s="9"/>
       <c r="N2" s="10">
         <f>SUM(C2:M2)</f>
-        <v>0</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="3" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="37"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="30"/>
+      <c r="A3" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="29">
+        <v>6.25E-2</v>
+      </c>
+      <c r="C3" s="30">
+        <v>6.25E-2</v>
+      </c>
       <c r="D3" s="31"/>
       <c r="E3" s="30"/>
       <c r="F3" s="31"/>
@@ -3749,1785 +3713,88 @@
       <c r="M3" s="33"/>
       <c r="N3" s="10">
         <f>SUM(C3:M3)</f>
-        <v>0</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="4" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="38"/>
-      <c r="B4" s="29"/>
-      <c r="C4" s="30"/>
-      <c r="D4" s="34"/>
+      <c r="A4" s="37" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="29">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="C4" s="30">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D4" s="31"/>
       <c r="E4" s="30"/>
-      <c r="F4" s="34"/>
-      <c r="G4" s="30"/>
-      <c r="H4" s="34"/>
-      <c r="I4" s="30"/>
-      <c r="J4" s="34"/>
-      <c r="K4" s="34"/>
-      <c r="L4" s="30"/>
-      <c r="M4" s="35"/>
+      <c r="F4" s="31"/>
+      <c r="G4" s="32"/>
+      <c r="H4" s="31"/>
+      <c r="I4" s="31"/>
+      <c r="J4" s="31"/>
+      <c r="K4" s="31"/>
+      <c r="L4" s="31"/>
+      <c r="M4" s="33"/>
       <c r="N4" s="10">
         <f>SUM(C4:M4)</f>
-        <v>0</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="5" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="39"/>
-      <c r="B5" s="29"/>
-      <c r="C5" s="30"/>
-      <c r="D5" s="34"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="10">
-        <f t="shared" ref="N5:N13" si="0">SUM(C5:M5)</f>
-        <v>0</v>
-      </c>
+      <c r="A5" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" s="24"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="26"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="26"/>
+      <c r="G5" s="25"/>
+      <c r="H5" s="26"/>
+      <c r="I5" s="25"/>
+      <c r="J5" s="26"/>
+      <c r="K5" s="26"/>
+      <c r="L5" s="25"/>
+      <c r="M5" s="27"/>
+      <c r="N5" s="10"/>
     </row>
     <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="13"/>
+      <c r="A6" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="B6" s="29">
+        <v>6.25E-2</v>
+      </c>
+      <c r="C6" s="30">
+        <v>6.25E-2</v>
+      </c>
+      <c r="D6" s="34"/>
+      <c r="E6" s="30"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="30"/>
+      <c r="H6" s="34"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
+      <c r="L6" s="30"/>
+      <c r="M6" s="35"/>
       <c r="N6" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="37"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="12"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10"/>
-      <c r="L7" s="12"/>
-      <c r="M7" s="13"/>
-      <c r="N7" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="37"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
-      <c r="L8" s="12"/>
-      <c r="M8" s="13"/>
-      <c r="N8" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="37"/>
-      <c r="B9" s="11"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="12"/>
-      <c r="M9" s="13"/>
-      <c r="N9" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="37"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="14"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="14"/>
-      <c r="M10" s="13"/>
-      <c r="N10" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="37"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="14"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="14"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="14"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="14"/>
-      <c r="M11" s="13"/>
-      <c r="N11" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="37"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="13"/>
-      <c r="N12" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="37"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="14"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="10">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="38"/>
-      <c r="B14" s="29"/>
-      <c r="C14" s="31"/>
-      <c r="D14" s="34"/>
-      <c r="E14" s="31"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="31"/>
-      <c r="H14" s="34"/>
-      <c r="I14" s="31"/>
-      <c r="J14" s="34"/>
-      <c r="K14" s="34"/>
-      <c r="L14" s="31"/>
-      <c r="M14" s="35"/>
-      <c r="N14" s="10">
-        <f>SUM(C14:M14)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="37"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="14"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="13"/>
-      <c r="N15" s="10">
-        <f t="shared" ref="N15:N28" si="1">SUM(C15:M15)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="37"/>
-      <c r="B16" s="11"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="14"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="13"/>
-      <c r="N16" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="37"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="13"/>
-      <c r="N17" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="37"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10"/>
-      <c r="L18" s="12"/>
-      <c r="M18" s="13"/>
-      <c r="N18" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="37"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="10"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10"/>
-      <c r="L19" s="12"/>
-      <c r="M19" s="13"/>
-      <c r="N19" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="37"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="12"/>
-      <c r="M20" s="13"/>
-      <c r="N20" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="37"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="10"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10"/>
-      <c r="L21" s="12"/>
-      <c r="M21" s="13"/>
-      <c r="N21" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="37"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="10"/>
-      <c r="I22" s="12"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10"/>
-      <c r="L22" s="12"/>
-      <c r="M22" s="13"/>
-      <c r="N22" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="37"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="10"/>
-      <c r="I23" s="12"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10"/>
-      <c r="L23" s="12"/>
-      <c r="M23" s="13"/>
-      <c r="N23" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="37"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="12"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10"/>
-      <c r="L24" s="12"/>
-      <c r="M24" s="13"/>
-      <c r="N24" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="37"/>
-      <c r="B25" s="11"/>
-      <c r="C25" s="14"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="14"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="14"/>
-      <c r="H25" s="10"/>
-      <c r="I25" s="12"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10"/>
-      <c r="L25" s="12"/>
-      <c r="M25" s="13"/>
-      <c r="N25" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="37"/>
-      <c r="B26" s="11"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-      <c r="M26" s="13"/>
-      <c r="N26" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="37"/>
-      <c r="B27" s="11"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
-      <c r="I27" s="12"/>
-      <c r="J27" s="12"/>
-      <c r="K27" s="12"/>
-      <c r="L27" s="12"/>
-      <c r="M27" s="16"/>
-      <c r="N27" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="40"/>
-      <c r="B28" s="17"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="20"/>
-      <c r="M28" s="21"/>
-      <c r="N28" s="10">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B29" s="10">
-        <f t="shared" ref="B29:M29" si="2">SUM(B2:B28)</f>
-        <v>0</v>
-      </c>
-      <c r="C29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="D29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="E29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="F29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="G29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="H29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="I29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="J29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="K29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="L29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="M29" s="10">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M30" s="10">
-        <f>SUM(C29:M29)</f>
-        <v>0</v>
-      </c>
-      <c r="N30" s="10">
-        <f>SUM(N2:N28)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="52" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="53" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="54" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="55" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="56" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="57" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="58" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="59" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="60" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="61" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="62" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="63" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="64" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="65" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="66" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="67" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="68" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="69" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="70" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="71" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="72" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="73" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="74" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="75" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="76" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="77" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="78" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="79" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="80" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="81" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="82" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="83" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="84" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="85" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="86" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="87" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="88" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="89" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="90" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="91" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="92" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="93" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="94" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="103" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="104" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="105" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="106" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="107" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="108" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="109" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="110" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="111" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="112" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="113" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="114" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="115" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="116" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="117" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="118" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="119" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="120" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="121" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="122" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="123" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="124" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="125" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="126" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="127" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="128" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="129" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="130" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="131" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="132" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="133" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="134" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="135" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="136" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="137" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="138" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="139" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="140" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="141" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="142" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="143" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="144" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="145" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="146" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="147" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="148" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="149" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="150" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="151" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="152" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="153" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="154" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="155" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="156" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="157" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="158" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="159" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="160" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="161" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="162" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="163" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="164" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="165" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="166" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="167" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="168" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="169" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="170" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="171" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="172" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="173" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="174" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="175" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="176" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="177" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="178" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="179" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="180" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="181" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="182" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="183" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="184" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="185" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="186" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="187" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="188" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="189" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="190" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="191" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="192" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="193" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="194" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="195" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="196" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="197" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="198" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="199" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="200" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="201" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="202" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="203" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="204" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="205" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="206" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="207" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="208" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="209" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="210" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="211" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="212" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="213" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="214" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="215" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="216" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="217" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="218" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="219" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="220" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="221" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="222" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="223" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="224" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="225" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="226" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="227" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="228" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="229" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="230" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="231" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="232" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="233" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="234" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="235" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="236" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="237" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="238" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="239" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="240" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="241" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="242" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="243" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="244" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="245" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="246" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="247" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="248" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="249" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="250" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="251" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="252" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="253" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="254" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="255" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="256" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="257" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="258" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="259" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="260" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="261" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="262" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="263" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="264" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="265" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="266" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="267" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="268" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="269" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="270" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="271" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="272" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="273" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="274" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="275" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="276" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="277" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="278" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="279" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="280" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="281" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="282" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="283" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="284" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="285" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="286" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="287" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="288" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="289" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="290" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="291" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="292" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="293" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="294" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="295" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="296" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="297" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="298" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="299" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="300" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="301" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="302" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="303" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="304" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="305" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="306" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="307" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="308" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="309" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="310" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="311" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="312" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="313" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="314" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="315" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="316" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="317" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="318" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="319" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="320" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="321" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="322" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="323" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="324" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="325" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="326" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="327" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="328" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="329" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="330" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="331" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="332" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="333" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="334" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="335" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="336" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="337" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="338" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="339" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="340" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="341" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="342" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="343" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="344" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="345" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="346" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="347" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="348" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="349" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="350" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="351" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="352" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="353" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="354" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="355" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="356" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="357" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="358" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="359" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="360" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="361" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="362" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="363" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="364" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="365" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="366" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="367" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="368" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="369" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="370" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="371" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="372" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="373" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="374" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="375" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="376" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="377" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="378" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="379" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="380" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="381" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="382" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="383" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="384" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="385" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="386" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="387" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="388" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="389" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="390" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="391" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="392" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="393" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="394" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="395" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="396" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="397" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="398" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="399" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="400" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="401" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="402" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="403" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="404" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="405" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="406" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="407" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="408" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="409" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="410" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="411" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="412" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="413" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="414" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="415" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="416" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="417" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="418" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="419" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="420" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="421" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="422" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="423" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="424" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="425" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="426" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="427" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="428" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="429" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="430" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="431" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="432" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="433" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="434" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="435" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="436" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="437" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="438" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="439" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="440" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="441" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="442" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="443" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="444" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="445" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="446" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="447" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="448" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="449" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="450" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="451" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="452" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="453" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="454" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="455" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="456" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="457" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="458" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="459" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="460" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="461" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="462" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="463" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="464" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="465" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="466" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="467" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="468" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="469" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="470" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="471" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="472" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="473" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="474" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="475" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="476" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="477" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="478" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="479" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="480" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="481" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="482" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="483" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="484" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="485" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="486" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="487" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="488" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="489" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="490" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="491" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="492" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="493" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="494" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="495" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="496" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="497" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="498" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="499" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="500" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="501" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="502" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="503" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="504" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="505" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="506" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="507" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="508" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="509" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="510" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="511" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="512" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="513" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="514" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="515" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="516" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="517" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="518" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="519" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="520" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="521" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="522" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="523" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="524" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="525" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="526" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="527" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="528" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="529" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="530" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="531" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="532" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="533" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="534" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="535" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="536" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="537" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="538" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="539" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="540" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="541" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="542" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="543" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="544" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="545" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="546" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="547" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="548" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="549" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="550" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="551" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="552" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="553" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="554" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="555" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="556" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="557" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="558" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="559" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="560" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="561" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="562" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="563" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="564" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="565" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="566" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="567" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="568" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="569" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="570" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="571" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="572" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="573" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="574" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="575" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="576" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="577" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="578" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="579" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="580" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="581" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="582" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="583" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="584" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="585" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="586" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="587" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="588" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="589" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="590" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="591" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="592" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="593" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="594" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="595" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="596" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="597" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="598" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="599" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="600" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="601" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="602" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="603" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="604" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="605" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="606" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="607" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="608" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="609" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="610" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="611" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="612" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="613" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="614" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="615" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="616" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="617" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="618" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="619" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="620" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="621" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="622" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="623" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="624" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="625" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="626" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="627" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="628" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="629" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="630" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="631" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="632" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="633" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="634" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="635" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="636" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="637" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="638" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="639" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="640" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="641" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="642" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="643" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="644" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="645" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="646" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="647" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="648" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="649" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="650" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="651" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="652" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="653" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="654" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="655" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="656" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="657" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="658" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="659" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="660" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="661" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="662" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="663" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="664" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="665" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="666" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="667" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="668" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="669" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="670" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="671" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="672" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="673" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="674" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="675" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="676" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="677" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="678" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="679" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="680" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="681" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="682" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="683" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="684" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="685" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="686" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="687" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="688" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="689" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="690" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="691" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="692" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="693" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="694" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="695" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="696" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="697" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="698" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="699" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="700" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="701" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="702" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="703" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="704" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="705" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="706" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="707" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="708" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="709" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="710" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="711" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="712" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="713" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="714" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="715" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="716" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="717" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="718" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="719" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="720" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="721" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="722" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="723" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="724" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="725" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="726" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="727" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="728" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="729" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="730" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="731" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="732" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="733" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="734" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="735" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="736" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="737" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="738" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="739" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="740" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="741" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="742" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="743" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="744" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="745" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="746" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="747" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="748" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="749" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="750" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="751" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="752" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="753" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="754" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="755" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="756" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="757" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="758" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="759" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="760" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="761" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="762" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="763" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="764" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="765" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="766" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="767" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="768" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="769" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="770" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="771" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="772" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="773" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="774" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="775" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="776" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="777" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="778" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="779" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="780" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="781" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="782" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="783" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="784" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="785" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="786" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="787" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="788" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="789" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="790" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="791" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="792" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="793" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="794" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="795" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="796" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="797" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="798" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="799" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="800" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="801" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="802" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="803" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="804" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="805" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="806" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="807" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="808" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="809" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="810" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="811" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="812" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="813" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="814" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="815" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="816" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="817" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="818" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="819" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="820" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="821" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="822" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="823" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="824" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="825" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="826" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="827" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="828" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="829" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="830" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="831" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="832" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="833" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="834" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="835" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="836" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="837" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="838" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="839" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="840" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="841" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="842" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="843" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="844" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="845" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="846" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="847" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="848" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="849" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="850" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="851" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="852" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="853" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="854" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="855" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="856" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="857" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="858" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="859" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="860" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="861" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="862" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="863" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="864" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="865" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="866" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="867" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="868" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="869" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="870" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="871" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="872" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="873" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="874" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="875" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="876" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="877" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="878" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="879" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="880" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="881" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="882" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="883" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="884" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="885" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="886" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="887" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="888" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="889" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="890" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="891" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="892" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="893" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="894" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="895" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="896" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="897" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="898" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="899" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="900" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="901" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="902" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="903" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="904" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="905" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="906" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="907" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="908" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="909" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="910" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="911" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="912" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="913" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="914" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="915" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="916" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="917" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="918" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="919" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="920" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="921" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="922" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="923" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="924" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="925" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="926" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="927" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="928" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="929" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="930" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="931" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="932" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="933" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="934" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="935" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="936" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="937" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="938" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="939" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="940" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="941" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="942" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="943" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="944" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="945" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="946" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="947" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="948" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="949" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="950" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="951" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="952" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="953" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="954" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="955" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="956" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="957" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="958" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="959" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="960" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="961" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="962" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="963" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="964" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="965" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="966" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="967" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="968" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="969" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="970" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="971" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="972" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="973" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="974" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="975" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="976" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="977" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="978" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="979" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="980" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="981" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="982" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="983" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="984" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="985" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="986" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="987" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="988" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="989" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="990" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="991" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="992" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="993" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="994" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="995" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="996" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="997" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="998" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="999" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1000" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1001" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1002" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-  </sheetData>
-  <conditionalFormatting sqref="C2:J28 L2:M28">
-    <cfRule type="cellIs" dxfId="38" priority="23" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="37" priority="24" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="25" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:J13 L6:M13 C15:J28 L15:M28">
-    <cfRule type="cellIs" dxfId="35" priority="18" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:M3 K6:K13 K15:K28">
-    <cfRule type="cellIs" dxfId="34" priority="10" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:M3">
-    <cfRule type="cellIs" dxfId="33" priority="9" operator="greaterThan">
-      <formula>0.00001157407407</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C29:M29">
-    <cfRule type="cellIs" dxfId="32" priority="3" operator="equal">
-      <formula>0.333333333333333</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D26:D27 J26:J27 F27 H27 M27">
-    <cfRule type="cellIs" dxfId="31" priority="21" operator="greaterThan">
-      <formula>0.00001157407407</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G26">
-    <cfRule type="cellIs" dxfId="30" priority="22" operator="greaterThan">
-      <formula>0.00001157407407</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I25 C4:C28 E4:E28 G4:G28 L4:L28 F26 H26:I26 I27:I28">
-    <cfRule type="cellIs" dxfId="29" priority="17" operator="greaterThan">
-      <formula>0.00001157407407</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K28">
-    <cfRule type="cellIs" dxfId="28" priority="14" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="27" priority="15" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="16" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K26:K27">
-    <cfRule type="cellIs" dxfId="25" priority="12" operator="greaterThan">
-      <formula>0.00001157407407</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N28">
-    <cfRule type="cellIs" dxfId="24" priority="1" operator="equal">
-      <formula>$B2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AA1003"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="42.625" customWidth="1"/>
-    <col min="2" max="2" width="11.375" customWidth="1"/>
-    <col min="3" max="27" width="10" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="L1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="M1" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="O1" s="5"/>
-      <c r="P1" s="5"/>
-      <c r="Q1" s="5"/>
-      <c r="R1" s="5"/>
-      <c r="S1" s="5"/>
-      <c r="T1" s="5"/>
-      <c r="U1" s="5"/>
-      <c r="V1" s="5"/>
-      <c r="W1" s="5"/>
-      <c r="X1" s="5"/>
-      <c r="Y1" s="5"/>
-      <c r="Z1" s="5"/>
-      <c r="AA1" s="5"/>
-    </row>
-    <row r="2" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="36" t="s">
-        <v>35</v>
-      </c>
-      <c r="B2" s="6">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C2" s="7">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="D2" s="8"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="8"/>
-      <c r="I2" s="8"/>
-      <c r="J2" s="8"/>
-      <c r="K2" s="8"/>
-      <c r="L2" s="8"/>
-      <c r="M2" s="9"/>
-      <c r="N2" s="10">
-        <f>SUM(C2:M2)</f>
-        <v>4.1666666666666664E-2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="37" t="s">
-        <v>37</v>
-      </c>
-      <c r="B3" s="29">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C3" s="30">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="D3" s="31"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="32"/>
-      <c r="H3" s="31"/>
-      <c r="I3" s="31"/>
-      <c r="J3" s="31"/>
-      <c r="K3" s="31"/>
-      <c r="L3" s="31"/>
-      <c r="M3" s="33"/>
-      <c r="N3" s="10">
-        <f>SUM(C3:M3)</f>
-        <v>4.1666666666666664E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="23" t="s">
-        <v>38</v>
-      </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="25"/>
-      <c r="H4" s="26"/>
-      <c r="I4" s="25"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="25"/>
-      <c r="M4" s="27"/>
-      <c r="N4" s="10"/>
-    </row>
-    <row r="5" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="39" t="s">
-        <v>36</v>
-      </c>
-      <c r="B5" s="29">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="C5" s="30">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="D5" s="34"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="34"/>
-      <c r="G5" s="30"/>
-      <c r="H5" s="34"/>
-      <c r="I5" s="30"/>
-      <c r="J5" s="34"/>
-      <c r="K5" s="34"/>
-      <c r="L5" s="30"/>
-      <c r="M5" s="35"/>
-      <c r="N5" s="10">
-        <f t="shared" ref="N5:N13" si="0">SUM(C5:M5)</f>
-        <v>8.3333333333333329E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="37" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="11">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="C6" s="12">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="12"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10"/>
-      <c r="L6" s="12"/>
-      <c r="M6" s="13"/>
-      <c r="N6" s="10">
-        <f t="shared" si="0"/>
-        <v>4.1666666666666664E-2</v>
+        <f t="shared" ref="N6:N12" si="0">SUM(C6:M6)</f>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="7" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="37" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="11">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="12"/>
+      <c r="D7" s="10">
         <v>2.0833333333333332E-2</v>
       </c>
-      <c r="D7" s="10"/>
       <c r="E7" s="12"/>
       <c r="F7" s="10"/>
       <c r="G7" s="12"/>
@@ -5544,16 +3811,13 @@
     </row>
     <row r="8" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="37" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B8" s="11">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="C8" s="12">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="D8" s="10">
-        <v>4.1666666666666664E-2</v>
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="D8" s="12">
+        <v>2.0833333333333332E-2</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="10"/>
@@ -5565,22 +3829,21 @@
       <c r="L8" s="12"/>
       <c r="M8" s="13"/>
       <c r="N8" s="10">
-        <f t="shared" si="0"/>
-        <v>8.3333333333333329E-2</v>
+        <f>SUM(D8:M8)</f>
+        <v>2.0833333333333332E-2</v>
       </c>
     </row>
     <row r="9" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="37" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="B9" s="11">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="C9" s="12"/>
-      <c r="D9" s="10">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="E9" s="12"/>
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
       <c r="F9" s="10"/>
       <c r="G9" s="12"/>
       <c r="H9" s="10"/>
@@ -5590,46 +3853,44 @@
       <c r="L9" s="12"/>
       <c r="M9" s="13"/>
       <c r="N9" s="10">
-        <f>SUM(C9:M9)</f>
-        <v>8.3333333333333329E-2</v>
+        <f>SUM(D9:M9)</f>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="10" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="37" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B10" s="11">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="C10" s="14"/>
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="C10" s="12"/>
       <c r="D10" s="10">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="E10" s="14"/>
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E10" s="12"/>
       <c r="F10" s="10"/>
-      <c r="G10" s="14"/>
+      <c r="G10" s="12"/>
       <c r="H10" s="10"/>
-      <c r="I10" s="14"/>
+      <c r="I10" s="12"/>
       <c r="J10" s="10"/>
       <c r="K10" s="10"/>
-      <c r="L10" s="14"/>
+      <c r="L10" s="12"/>
       <c r="M10" s="13"/>
       <c r="N10" s="10">
         <f t="shared" si="0"/>
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="11" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="37" t="s">
-        <v>19</v>
+        <v>46</v>
       </c>
       <c r="B11" s="11">
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C11" s="14"/>
-      <c r="D11" s="10">
-        <v>4.1666666666666664E-2</v>
-      </c>
+      <c r="D11" s="10"/>
       <c r="E11" s="12">
         <v>4.1666666666666664E-2</v>
       </c>
@@ -5643,21 +3904,21 @@
       <c r="M11" s="13"/>
       <c r="N11" s="10">
         <f t="shared" si="0"/>
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="12" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="37" t="s">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="B12" s="11">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="C12" s="14"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="12">
-        <v>0.10416666666666667</v>
-      </c>
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="10">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E12" s="12"/>
       <c r="F12" s="10"/>
       <c r="G12" s="14"/>
       <c r="H12" s="10"/>
@@ -5668,66 +3929,66 @@
       <c r="M12" s="13"/>
       <c r="N12" s="10">
         <f t="shared" si="0"/>
-        <v>0.10416666666666667</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="13" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="37" t="s">
-        <v>21</v>
-      </c>
-      <c r="B13" s="11">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="12">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="F13" s="10"/>
-      <c r="G13" s="14"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="14"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="14"/>
-      <c r="M13" s="13"/>
-      <c r="N13" s="10">
-        <f t="shared" si="0"/>
-        <v>0.10416666666666667</v>
-      </c>
+      <c r="A13" s="23" t="s">
+        <v>23</v>
+      </c>
+      <c r="B13" s="24"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="28"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="28"/>
+      <c r="H13" s="26"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="26"/>
+      <c r="K13" s="26"/>
+      <c r="L13" s="28"/>
+      <c r="M13" s="27"/>
+      <c r="N13" s="10"/>
     </row>
     <row r="14" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="B14" s="24"/>
-      <c r="C14" s="28"/>
-      <c r="D14" s="26"/>
-      <c r="E14" s="28"/>
-      <c r="F14" s="26"/>
-      <c r="G14" s="28"/>
-      <c r="H14" s="26"/>
-      <c r="I14" s="28"/>
-      <c r="J14" s="26"/>
-      <c r="K14" s="26"/>
-      <c r="L14" s="28"/>
-      <c r="M14" s="27"/>
-      <c r="N14" s="10"/>
+      <c r="A14" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="11">
+        <v>6.25E-2</v>
+      </c>
+      <c r="C14" s="14"/>
+      <c r="D14" s="10">
+        <v>6.25E-2</v>
+      </c>
+      <c r="E14" s="12"/>
+      <c r="F14" s="10"/>
+      <c r="G14" s="14"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="14"/>
+      <c r="J14" s="10"/>
+      <c r="K14" s="10"/>
+      <c r="L14" s="14"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="10">
+        <f>SUM(C14:M14)</f>
+        <v>6.25E-2</v>
+      </c>
     </row>
     <row r="15" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="37" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B15" s="11">
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="10"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="10">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="G15" s="14"/>
+      <c r="E15" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F15" s="10"/>
+      <c r="G15" s="15"/>
       <c r="H15" s="10"/>
       <c r="I15" s="14"/>
       <c r="J15" s="10"/>
@@ -5735,24 +3996,24 @@
       <c r="L15" s="14"/>
       <c r="M15" s="13"/>
       <c r="N15" s="10">
-        <f t="shared" ref="N15:N29" si="1">SUM(C15:M15)</f>
-        <v>8.3333333333333329E-2</v>
+        <f t="shared" ref="N15:N38" si="1">SUM(C15:M15)</f>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="16" spans="1:27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="37" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="B16" s="11">
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C16" s="14"/>
       <c r="D16" s="10"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="10">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="G16" s="15"/>
+      <c r="E16" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F16" s="10"/>
+      <c r="G16" s="12"/>
       <c r="H16" s="10"/>
       <c r="I16" s="14"/>
       <c r="J16" s="10"/>
@@ -5761,50 +4022,47 @@
       <c r="M16" s="13"/>
       <c r="N16" s="10">
         <f t="shared" si="1"/>
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="37" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B17" s="11">
-        <v>0.125</v>
-      </c>
-      <c r="C17" s="14"/>
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="C17" s="12"/>
       <c r="D17" s="10"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="10">
-        <v>6.25E-2</v>
-      </c>
-      <c r="G17" s="12">
-        <v>6.25E-2</v>
-      </c>
+      <c r="E17" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="F17" s="10"/>
+      <c r="G17" s="12"/>
       <c r="H17" s="10"/>
-      <c r="I17" s="14"/>
+      <c r="I17" s="12"/>
       <c r="J17" s="10"/>
       <c r="K17" s="10"/>
-      <c r="L17" s="14"/>
+      <c r="L17" s="12"/>
       <c r="M17" s="13"/>
       <c r="N17" s="10">
         <f t="shared" si="1"/>
-        <v>0.125</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="37" t="s">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="B18" s="11">
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C18" s="12"/>
       <c r="D18" s="10"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="12">
-        <v>8.3333333333333329E-2</v>
-      </c>
+      <c r="F18" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="G18" s="12"/>
       <c r="H18" s="10"/>
       <c r="I18" s="12"/>
       <c r="J18" s="10"/>
@@ -5813,23 +4071,22 @@
       <c r="M18" s="13"/>
       <c r="N18" s="10">
         <f t="shared" si="1"/>
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="37" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="B19" s="11">
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="C19" s="12"/>
       <c r="D19" s="10"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="12">
-        <v>8.3333333333333329E-2</v>
-      </c>
+      <c r="F19" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="G19" s="12"/>
       <c r="H19" s="10"/>
       <c r="I19" s="12"/>
       <c r="J19" s="10"/>
@@ -5838,24 +4095,23 @@
       <c r="M19" s="13"/>
       <c r="N19" s="10">
         <f t="shared" si="1"/>
-        <v>8.3333333333333329E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="37" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B20" s="11">
         <v>4.1666666666666664E-2</v>
       </c>
       <c r="C20" s="12"/>
       <c r="D20" s="10"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="10">
-        <v>4.1666666666666664E-2</v>
-      </c>
+      <c r="F20" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
       <c r="I20" s="12"/>
       <c r="J20" s="10"/>
       <c r="K20" s="10"/>
@@ -5868,333 +4124,563 @@
     </row>
     <row r="21" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="37" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="11">
-        <v>2.0833333333333332E-2</v>
+        <v>33</v>
+      </c>
+      <c r="B21" s="29">
+        <v>0.125</v>
       </c>
       <c r="C21" s="12"/>
       <c r="D21" s="10"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="10"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="12"/>
-      <c r="H21" s="10">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="I21" s="12"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="12">
+        <v>0.125</v>
+      </c>
       <c r="J21" s="10"/>
       <c r="K21" s="10"/>
       <c r="L21" s="12"/>
-      <c r="M21" s="13"/>
+      <c r="M21" s="35"/>
       <c r="N21" s="10">
-        <f t="shared" si="1"/>
-        <v>2.0833333333333332E-2</v>
+        <f>SUM(C21:M21)</f>
+        <v>0.125</v>
       </c>
     </row>
     <row r="22" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="37" t="s">
-        <v>29</v>
-      </c>
-      <c r="B22" s="11">
-        <v>8.3333333333333329E-2</v>
+        <v>35</v>
+      </c>
+      <c r="B22" s="29">
+        <v>0.10416666666666667</v>
       </c>
       <c r="C22" s="12"/>
       <c r="D22" s="10"/>
       <c r="E22" s="12"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="12"/>
+      <c r="G22" s="10"/>
       <c r="H22" s="10">
-        <v>8.3333333333333329E-2</v>
+        <v>0.10416666666666667</v>
       </c>
       <c r="I22" s="12"/>
       <c r="J22" s="10"/>
       <c r="K22" s="10"/>
       <c r="L22" s="12"/>
-      <c r="M22" s="13"/>
+      <c r="M22" s="35"/>
       <c r="N22" s="10">
         <f t="shared" si="1"/>
-        <v>8.3333333333333329E-2</v>
+        <v>0.10416666666666667</v>
       </c>
     </row>
     <row r="23" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="37" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="11">
-        <v>0.10416666666666667</v>
+        <v>34</v>
+      </c>
+      <c r="B23" s="29">
+        <v>0.125</v>
       </c>
       <c r="C23" s="12"/>
       <c r="D23" s="10"/>
       <c r="E23" s="12"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="12"/>
+      <c r="G23" s="10">
+        <v>0.125</v>
+      </c>
       <c r="H23" s="10"/>
-      <c r="I23" s="12">
-        <v>0.10416666666666667</v>
-      </c>
+      <c r="I23" s="12"/>
       <c r="J23" s="10"/>
       <c r="K23" s="10"/>
       <c r="L23" s="12"/>
-      <c r="M23" s="13"/>
+      <c r="M23" s="35"/>
       <c r="N23" s="10">
         <f t="shared" si="1"/>
-        <v>0.10416666666666667</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="37" t="s">
-        <v>31</v>
-      </c>
-      <c r="B24" s="11">
-        <v>0.125</v>
+        <v>37</v>
+      </c>
+      <c r="B24" s="29">
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="C24" s="12"/>
       <c r="D24" s="10"/>
       <c r="E24" s="12"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="10"/>
-      <c r="I24" s="12">
-        <v>6.25E-2</v>
-      </c>
-      <c r="J24" s="10">
-        <v>6.25E-2</v>
-      </c>
+      <c r="F24" s="10">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="G24" s="10"/>
+      <c r="H24" s="12"/>
+      <c r="I24" s="12"/>
+      <c r="J24" s="10"/>
       <c r="K24" s="10"/>
       <c r="L24" s="12"/>
-      <c r="M24" s="13"/>
+      <c r="M24" s="35"/>
       <c r="N24" s="10">
         <f t="shared" si="1"/>
-        <v>0.125</v>
+        <v>8.3333333333333329E-2</v>
       </c>
     </row>
     <row r="25" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="37" t="s">
-        <v>32</v>
-      </c>
-      <c r="B25" s="11">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="C25" s="14"/>
+        <v>36</v>
+      </c>
+      <c r="B25" s="29">
+        <v>6.25E-2</v>
+      </c>
+      <c r="C25" s="12"/>
       <c r="D25" s="10"/>
-      <c r="E25" s="14"/>
+      <c r="E25" s="12"/>
       <c r="F25" s="10"/>
-      <c r="G25" s="14"/>
+      <c r="G25" s="12">
+        <v>6.25E-2</v>
+      </c>
       <c r="H25" s="10"/>
       <c r="I25" s="12"/>
-      <c r="J25" s="10">
-        <v>8.3333333333333329E-2</v>
-      </c>
+      <c r="J25" s="10"/>
       <c r="K25" s="10"/>
       <c r="L25" s="12"/>
-      <c r="M25" s="13"/>
+      <c r="M25" s="35"/>
       <c r="N25" s="10">
         <f t="shared" si="1"/>
-        <v>8.3333333333333329E-2</v>
+        <v>6.25E-2</v>
       </c>
     </row>
     <row r="26" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="B26" s="24"/>
-      <c r="C26" s="28"/>
-      <c r="D26" s="26"/>
-      <c r="E26" s="28"/>
-      <c r="F26" s="26"/>
-      <c r="G26" s="28"/>
-      <c r="H26" s="26"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="26"/>
-      <c r="K26" s="26"/>
-      <c r="L26" s="28"/>
-      <c r="M26" s="27"/>
-      <c r="N26" s="10"/>
+      <c r="A26" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="B26" s="29">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C26" s="12"/>
+      <c r="D26" s="10"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="10"/>
+      <c r="G26" s="40"/>
+      <c r="H26" s="12"/>
+      <c r="I26" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="12"/>
+      <c r="M26" s="35"/>
+      <c r="N26" s="10">
+        <f t="shared" si="1"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
     </row>
     <row r="27" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="37" t="s">
-        <v>41</v>
-      </c>
-      <c r="B27" s="11">
-        <v>0.47916666666666669</v>
+        <v>39</v>
+      </c>
+      <c r="B27" s="29">
+        <v>8.3333333333333329E-2</v>
       </c>
       <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
+      <c r="D27" s="10"/>
       <c r="E27" s="12"/>
-      <c r="F27" s="12">
-        <v>2.0833333333333332E-2</v>
-      </c>
-      <c r="G27" s="12">
-        <v>4.1666666666666664E-2</v>
-      </c>
-      <c r="H27" s="12">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="I27" s="12">
-        <v>6.25E-2</v>
-      </c>
-      <c r="J27" s="12">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="K27" s="12">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="L27" s="12">
-        <v>6.25E-2</v>
-      </c>
-      <c r="M27" s="13"/>
+      <c r="F27" s="10"/>
+      <c r="G27" s="12"/>
+      <c r="J27" s="10">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="K27" s="10"/>
+      <c r="L27" s="12"/>
+      <c r="M27" s="35"/>
       <c r="N27" s="10">
         <f t="shared" si="1"/>
-        <v>0.47916666666666669</v>
+        <v>8.3333333333333329E-2</v>
       </c>
     </row>
     <row r="28" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="37" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B28" s="11">
-        <v>1.25</v>
-      </c>
-      <c r="C28" s="12">
-        <v>6.25E-2</v>
-      </c>
-      <c r="D28" s="12">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="E28" s="12">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="F28" s="12">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="G28" s="12">
-        <v>6.25E-2</v>
-      </c>
-      <c r="H28" s="12">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="I28" s="12">
-        <v>0.10416666666666667</v>
-      </c>
-      <c r="J28" s="12">
-        <v>8.3333333333333329E-2</v>
-      </c>
-      <c r="K28" s="12">
-        <v>0.22916666666666666</v>
-      </c>
-      <c r="L28" s="12">
-        <v>0.27083333333333331</v>
-      </c>
-      <c r="M28" s="16">
-        <v>8.3333333333333329E-2</v>
-      </c>
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C28" s="12"/>
+      <c r="D28" s="10"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="10"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="10"/>
+      <c r="J28" s="10">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="K28" s="10"/>
+      <c r="L28" s="12"/>
+      <c r="M28" s="13"/>
       <c r="N28" s="10">
         <f t="shared" si="1"/>
-        <v>1.2499999999999998</v>
+        <v>8.3333333333333329E-2</v>
       </c>
     </row>
     <row r="29" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="40" t="s">
-        <v>34</v>
-      </c>
-      <c r="B29" s="17">
-        <v>0.25</v>
-      </c>
-      <c r="C29" s="18"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="18"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="19"/>
-      <c r="L29" s="20"/>
-      <c r="M29" s="21">
-        <v>0.25</v>
-      </c>
+      <c r="A29" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="B29" s="11">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C29" s="12"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="10"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="10"/>
+      <c r="J29" s="10">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="K29" s="12"/>
+      <c r="L29" s="12"/>
+      <c r="M29" s="13"/>
       <c r="N29" s="10">
         <f t="shared" si="1"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="37" t="s">
+        <v>42</v>
+      </c>
+      <c r="B30" s="29">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C30" s="12"/>
+      <c r="D30" s="10"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="10"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="12"/>
+      <c r="J30" s="10">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="K30" s="10">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="L30" s="12"/>
+      <c r="M30" s="35"/>
+      <c r="N30" s="10">
+        <f t="shared" si="1"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="37" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" s="29">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C31" s="12"/>
+      <c r="D31" s="10"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="10"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="10"/>
+      <c r="K31" s="10">
+        <v>8.3333333333333301E-2</v>
+      </c>
+      <c r="L31" s="10"/>
+      <c r="M31" s="35"/>
+      <c r="N31" s="10">
+        <f t="shared" si="1"/>
+        <v>8.3333333333333301E-2</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="37" t="s">
+        <v>44</v>
+      </c>
+      <c r="B32" s="29">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="C32" s="12"/>
+      <c r="D32" s="10"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="10"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="12"/>
+      <c r="K32" s="10">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="L32" s="10"/>
+      <c r="M32" s="35"/>
+      <c r="N32" s="10">
+        <f t="shared" si="1"/>
+        <v>8.3333333333333329E-2</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="37" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="29">
+        <v>0.10416666666666667</v>
+      </c>
+      <c r="C33" s="12"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="10"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="12"/>
+      <c r="L33" s="10">
+        <v>0.10416666666666667</v>
+      </c>
+      <c r="M33" s="35"/>
+      <c r="N33" s="10">
+        <f>SUM(C33:M33)</f>
+        <v>0.10416666666666667</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="B34" s="24"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="26"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="26"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="26"/>
+      <c r="I34" s="28"/>
+      <c r="J34" s="26"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="28"/>
+      <c r="M34" s="27"/>
+      <c r="N34" s="10"/>
+    </row>
+    <row r="35" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="37" t="s">
+        <v>49</v>
+      </c>
+      <c r="B35" s="11">
+        <v>0.375</v>
+      </c>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="E35" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="F35" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="G35" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="H35" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="I35" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="J35" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="K35" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="L35" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="M35" s="13">
+        <v>0.125</v>
+      </c>
+      <c r="N35" s="10">
+        <f t="shared" si="1"/>
+        <v>0.375</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="37" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="11">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="30" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="10">
-        <f t="shared" ref="B30:M30" si="2">SUM(B2:B29)</f>
-        <v>3.6666666666666665</v>
-      </c>
-      <c r="C30" s="10">
+      <c r="C36" s="12">
+        <v>4.1666666666666664E-2</v>
+      </c>
+      <c r="D36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="E36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="F36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="G36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="H36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="I36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="J36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="K36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="L36" s="12">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="M36" s="13">
+        <v>2.0833333333333332E-2</v>
+      </c>
+      <c r="N36" s="10">
+        <f t="shared" si="1"/>
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="37" t="s">
+        <v>17</v>
+      </c>
+      <c r="B37" s="11">
+        <v>1</v>
+      </c>
+      <c r="C37" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="D37" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="E37" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="F37" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="G37" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="H37" s="12">
+        <v>0.16666666666666666</v>
+      </c>
+      <c r="I37" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12">
+        <v>8.3333333333333329E-2</v>
+      </c>
+      <c r="L37" s="12">
+        <v>0.1875</v>
+      </c>
+      <c r="M37" s="16">
+        <v>6.25E-2</v>
+      </c>
+      <c r="N37" s="10">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" ht="14.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38" s="39" t="s">
+        <v>18</v>
+      </c>
+      <c r="B38" s="17">
+        <v>0.125</v>
+      </c>
+      <c r="C38" s="18"/>
+      <c r="D38" s="19"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="19"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="19"/>
+      <c r="I38" s="18"/>
+      <c r="J38" s="19"/>
+      <c r="K38" s="19"/>
+      <c r="L38" s="20"/>
+      <c r="M38" s="21">
+        <v>0.125</v>
+      </c>
+      <c r="N38" s="10">
+        <f t="shared" si="1"/>
+        <v>0.125</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B39" s="10">
+        <f t="shared" ref="B39:M39" si="2">SUM(B2:B38)</f>
+        <v>3.6666666666666661</v>
+      </c>
+      <c r="C39" s="10">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="D30" s="10">
+      <c r="D39" s="10">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="E30" s="10">
+      <c r="E39" s="10">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="F30" s="10">
+      <c r="F39" s="10">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="G30" s="10">
+      <c r="G39" s="10">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="H30" s="10">
+      <c r="H39" s="10">
+        <f t="shared" si="2"/>
+        <v>0.33333333333333337</v>
+      </c>
+      <c r="I39" s="10">
         <f t="shared" si="2"/>
         <v>0.33333333333333331</v>
       </c>
-      <c r="I30" s="10">
+      <c r="J39" s="10">
+        <f t="shared" si="2"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="K39" s="10">
+        <f t="shared" si="2"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="L39" s="10">
         <f t="shared" si="2"/>
         <v>0.33333333333333337</v>
       </c>
-      <c r="J30" s="10">
+      <c r="M39" s="10">
         <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="K30" s="10">
-        <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="L30" s="10">
-        <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
-      </c>
-      <c r="M30" s="10">
-        <f t="shared" si="2"/>
-        <v>0.33333333333333331</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="M31" s="10">
-        <f>SUM(C30:M30)</f>
-        <v>3.666666666666667</v>
-      </c>
-      <c r="N31" s="10">
-        <f>SUM(N2:N29)</f>
+        <v>0.33333333333333337</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="M40" s="10">
+        <f>SUM(C39:M39)</f>
+        <v>3.6666666666666674</v>
+      </c>
+      <c r="N40" s="10">
+        <f>SUM(N2:N38)</f>
         <v>3.6666666666666661</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="36" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="37" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="38" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="39" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="40" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="41" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="42" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="43" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="44" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="45" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="46" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="47" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="48" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="41" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="42" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="43" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="44" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="45" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="46" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="47" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="48" spans="1:14" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="49" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="50" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="51" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -7151,116 +5637,196 @@
     <row r="1002" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1003" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
-  <conditionalFormatting sqref="C24:J26 L24:M26">
-    <cfRule type="cellIs" dxfId="23" priority="5" operator="greaterThan">
+  <conditionalFormatting sqref="C5:C7 D8:D9 F18:F21 E22:E38 G24:H24 G25 H26 J27:J28 G27:G38 I30:I34 J29:K29">
+    <cfRule type="cellIs" dxfId="37" priority="40" operator="greaterThan">
+      <formula>0.00001157407407</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C7 D8 D9:J9 F18:J20 F21 C22:E23 C24:J25 C26:F26 H26:J26 C27:G27 C28:H29 K29 C30:J31 C32:I33 C34:K34 K5:M12 C14:J17 L14:M34 C18:D21 G21:J23 J27:J29">
+    <cfRule type="cellIs" dxfId="36" priority="39" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C26:J26 L26:M26">
-    <cfRule type="cellIs" dxfId="22" priority="6" operator="greaterThan">
+  <conditionalFormatting sqref="C37:D37">
+    <cfRule type="cellIs" dxfId="35" priority="36" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="7" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="34" priority="36" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="33" priority="36" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C27:J29 L27:M29">
-    <cfRule type="cellIs" dxfId="20" priority="28" operator="greaterThan">
+  <conditionalFormatting sqref="C5:J6 D7:J8">
+    <cfRule type="cellIs" dxfId="32" priority="34" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="29" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="31" priority="34" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="30" operator="greaterThan">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C10:J12">
+    <cfRule type="cellIs" dxfId="30" priority="31" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="29" priority="31" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="31" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C27:J29">
-    <cfRule type="cellIs" dxfId="17" priority="23" operator="greaterThan">
+  <conditionalFormatting sqref="C35:J36 L35:M38 E37:J37 L31:L33 C38:J38 G36:H37 K14:K32">
+    <cfRule type="cellIs" dxfId="27" priority="41" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:M3">
-    <cfRule type="cellIs" dxfId="16" priority="14" operator="greaterThan">
+  <conditionalFormatting sqref="C35:J36 L35:M38 E37:J37 G36:H37">
+    <cfRule type="cellIs" dxfId="26" priority="38" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C35:K35 C36:J36 E37:J37 C38:J38 K36:K38 L31:L33 G36:H37 K14:K32">
+    <cfRule type="cellIs" dxfId="25" priority="35" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:M4 K34:K38">
+    <cfRule type="cellIs" dxfId="24" priority="33" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C2:M4">
+    <cfRule type="cellIs" dxfId="23" priority="28" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="29" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:M25 K27:K29">
-    <cfRule type="cellIs" dxfId="15" priority="21" operator="greaterThan">
+  <conditionalFormatting sqref="C13:M13">
+    <cfRule type="cellIs" dxfId="21" priority="22" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="22" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="22" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:M25">
-    <cfRule type="cellIs" dxfId="14" priority="15" operator="greaterThan">
+  <conditionalFormatting sqref="C39:M39">
+    <cfRule type="cellIs" dxfId="18" priority="25" operator="equal">
+      <formula>0.333333333333333</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D35:D36 J35:J37 M37 F37:H37">
+    <cfRule type="cellIs" dxfId="17" priority="42" operator="greaterThan">
+      <formula>0.00001157407407</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D37">
+    <cfRule type="cellIs" dxfId="16" priority="18" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
+    <cfRule type="cellIs" dxfId="15" priority="18" operator="greaterThan">
+      <formula>0.00001157407407</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C30:M30">
-    <cfRule type="cellIs" dxfId="13" priority="8" operator="equal">
-      <formula>0.333333333333333</formula>
+  <conditionalFormatting sqref="D7:J8 C5:J6">
+    <cfRule type="cellIs" dxfId="14" priority="43" operator="greaterThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D27:D28 J27:J28 F28 H28 M28">
-    <cfRule type="cellIs" dxfId="12" priority="26" operator="greaterThan">
+  <conditionalFormatting sqref="E5:E17 G5:G23 I5:I26 L5:L38 C10:C38">
+    <cfRule type="cellIs" dxfId="13" priority="16" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F27 H27:I27 I28:I29">
-    <cfRule type="cellIs" dxfId="11" priority="22" operator="greaterThan">
+  <conditionalFormatting sqref="F35:F36 H35:I36 I37:I38">
+    <cfRule type="cellIs" dxfId="12" priority="44" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G27">
-    <cfRule type="cellIs" dxfId="10" priority="27" operator="greaterThan">
+  <conditionalFormatting sqref="G35:G36">
+    <cfRule type="cellIs" dxfId="11" priority="37" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I4:I26 C4:C29 E4:E29 G4:G29 L4:L29">
-    <cfRule type="cellIs" dxfId="9" priority="4" operator="greaterThan">
+  <conditionalFormatting sqref="L31:L33 C35:J36 L35:M38 E37:J37 C38:J38 G36:H37 K14:K32">
+    <cfRule type="cellIs" dxfId="10" priority="45" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K34:K38 C2:M4">
+    <cfRule type="cellIs" dxfId="9" priority="32" operator="greaterThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K35:K37">
+    <cfRule type="cellIs" dxfId="8" priority="30" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K26">
-    <cfRule type="cellIs" dxfId="8" priority="2" operator="greaterThan">
+  <conditionalFormatting sqref="K5:M12 C7 D8 D9:J9 C14:J17 L14:M34 F18:J20 C18:D21 F21 G21:J23 C22:E23 C24:J25 C26:F26 H26:J26 C27:G27 C28:H29 K29 C30:J31 C32:I33 C34:J34 J27:J29">
+    <cfRule type="cellIs" dxfId="7" priority="20" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="6" priority="21" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K26:K29">
-    <cfRule type="cellIs" dxfId="6" priority="1" operator="greaterThan">
+  <conditionalFormatting sqref="K35:M38">
+    <cfRule type="cellIs" dxfId="5" priority="46" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K27:K28">
-    <cfRule type="cellIs" dxfId="5" priority="17" operator="greaterThan">
+  <conditionalFormatting sqref="N2:N4 N6:N12 N14:N33">
+    <cfRule type="cellIs" dxfId="4" priority="27" operator="equal">
+      <formula>$B2</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N35:N38">
+    <cfRule type="cellIs" dxfId="3" priority="26" operator="equal">
+      <formula>$B35</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:XFD1048576">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color theme="4" tint="0.59999389629810485"/>
+        <color theme="8" tint="0.39997558519241921"/>
+        <color theme="8" tint="-0.249977111117893"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color theme="3" tint="0.59999389629810485"/>
+        <color theme="8" tint="0.39997558519241921"/>
+        <color theme="8" tint="-0.249977111117893"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H36:H37">
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="greaterThan">
       <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K27:K29 C2:M25">
-    <cfRule type="cellIs" dxfId="4" priority="20" operator="greaterThan">
-      <formula>0</formula>
+  <conditionalFormatting sqref="G36">
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="greaterThan">
+      <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K27:M29">
-    <cfRule type="cellIs" dxfId="3" priority="19" operator="greaterThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N3">
-    <cfRule type="cellIs" dxfId="2" priority="12" operator="equal">
-      <formula>$B2</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N5:N13">
-    <cfRule type="cellIs" dxfId="1" priority="11" operator="equal">
-      <formula>$B5</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N15:N25 N27:N29">
-    <cfRule type="cellIs" dxfId="0" priority="10" operator="equal">
-      <formula>$B15</formula>
+  <conditionalFormatting sqref="H36">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <formula>0.00001157407407</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>

</xml_diff>